<commit_message>
Align requirements backlog and prototype for first assessment
</commit_message>
<xml_diff>
--- a/ProductBacklog_group27_draft.xlsx
+++ b/ProductBacklog_group27_draft.xlsx
@@ -11,10 +11,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,6 +27,13 @@
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -71,7 +80,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -95,6 +104,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -352,7 +373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="1" min="1" max="1"/>
@@ -444,13 +465,13 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Maintain reusable applicant profile</t>
+          <t>Maintain detailed reusable applicant profile</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
           <t>As an applicant
-I want to create and maintain a reusable profile
+I want to create and maintain a detailed reusable profile with my identity, academic background, skills, experience, and availability
 So that I do not need to re-enter the same information every time I apply for a TA role.</t>
         </is>
       </c>
@@ -464,17 +485,18 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>1. The applicant must be able to create and edit a profile.
-2. The profile must be saved and reused across multiple applications.
-3. The system must validate required profile fields before saving.</t>
+          <t>1. The profile must include full name, student ID, email, phone number, degree/programme, and year of study.
+2. The profile must support relevant modules or grades, technical skills and tools, previous TA experience, project or leadership experience, and availability.
+3. The profile must be saved and reused across multiple applications.
+4. The system must validate required profile fields before saving.</t>
         </is>
       </c>
       <c r="H2" s="5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>Applicant requirement: reusable profile</t>
+          <t>Applicant requirement: detailed reusable profile</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
@@ -560,14 +582,14 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Browse available vacancies</t>
+          <t>Browse vacancies before login</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>As an applicant
-I want to browse available TA vacancies
-So that I can find suitable roles.</t>
+          <t>As a visitor
+I want to browse available TA vacancies before logging in
+So that I can explore suitable roles easily before deciding to sign in.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -580,9 +602,9 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>1. The system must show open vacancies to the applicant.
-2. Each vacancy must display key summary information.
-3. If there are no open vacancies, the system must show an appropriate message.</t>
+          <t>1. The system must show open vacancies to a visitor without requiring login first.
+2. Each vacancy must display key summary information such as title, module, required skills, and deadline.
+3. The public vacancy interface must include a visible Log In entry.</t>
         </is>
       </c>
       <c r="H4" s="5" t="n">
@@ -590,7 +612,7 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Applicant requirement: browse vacancies</t>
+          <t>Applicant requirement: public browsing before login</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
@@ -618,14 +640,14 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>View vacancy details</t>
+          <t>View vacancy details before login</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>As an applicant
-I want to view full vacancy details, including module name, duties, required skills, workload, and deadline
-So that I can decide whether to apply.</t>
+          <t>As a visitor
+I want to view full vacancy details before logging in
+So that I can decide whether the role is relevant before signing in.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -638,9 +660,9 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>1. The system must display module name, duties, required skills, workload, and deadline.
+          <t>1. The system must display module name, duties, required skills, workload, and deadline before login.
 2. The displayed details must match the stored vacancy record.
-3. The applicant must be able to open the details from the vacancy list.</t>
+3. The vacancy details page must provide a visible Log In entry and an application path after authentication.</t>
         </is>
       </c>
       <c r="H5" s="5" t="n">
@@ -648,7 +670,7 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Applicant requirement: clear vacancy details</t>
+          <t>Applicant requirement: public vacancy details</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -698,7 +720,8 @@
         <is>
           <t>1. The applicant must be able to submit an application for an open vacancy.
 2. The system must save the application using the applicant profile and CV reference.
-3. A new application must start with the status Submitted.</t>
+3. A new application must start with the status Submitted.
+4. If the user is not logged in, the system must prompt login before the application can be submitted.</t>
         </is>
       </c>
       <c r="H6" s="5" t="n">
@@ -734,14 +757,14 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Apply for multiple roles</t>
+          <t>Apply within configurable role limit</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
           <t>As an applicant
-I want to apply for more than one TA role
-So that I can increase my chances of being selected.</t>
+I want to apply for more than one TA role only within the current configured limit
+So that workload control is enforced before later manual balancing is needed.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -754,9 +777,9 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>1. The applicant must be able to submit applications to different vacancies.
-2. Each application must be stored separately.
-3. The system must preserve the status of each application independently.</t>
+          <t>1. The applicant must be able to submit applications to different vacancies until the current limit is reached.
+2. The system must stop new applications once the current max_workload limit is reached.
+3. The current limit must be visible where it affects applicant decisions.</t>
         </is>
       </c>
       <c r="H7" s="5" t="n">
@@ -764,7 +787,7 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Applicant requirement: multiple applications</t>
+          <t>Applicant requirement: configurable role limit</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -798,7 +821,7 @@
       <c r="D8" s="6" t="inlineStr">
         <is>
           <t>As an applicant
-I want to view the status of each application, such as Submitted, Accepted, or Rejected
+I want to view the status of each application, such as Submitted, Offered, or Unsuccessful
 So that I can track progress clearly.</t>
         </is>
       </c>
@@ -813,7 +836,7 @@
       <c r="G8" s="6" t="inlineStr">
         <is>
           <t>1. The applicant must be able to see all submitted applications.
-2. The system must display statuses such as Submitted, Accepted, and Rejected clearly.
+2. The system must display statuses such as Submitted, Offered, and Unsuccessful clearly.
 3. Status updates made by a module organiser must appear correctly to the applicant.</t>
         </is>
       </c>
@@ -1082,14 +1105,14 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Record accept/reject decision</t>
+          <t>Record offer or rejection outcome</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
           <t>As a module organiser
-I want to accept or reject applicants and record the decision in the system
-So that recruitment decisions are consistent and traceable.</t>
+I want to record whether an applicant is offered the role or is unsuccessful
+So that recruitment outcomes are consistent and traceable.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1102,7 +1125,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>1. The module organiser must be able to change an application to Accepted or Rejected.
+          <t>1. The module organiser must be able to change an application to Offered or Unsuccessful.
 2. The decision must be saved in the recruitment record.
 3. The applicant view must show the updated decision correctly.</t>
         </is>
@@ -1112,7 +1135,7 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>MO requirement: accept/reject and record decision</t>
+          <t>MO requirement: record recruitment outcome</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -1534,61 +1557,586 @@
       </c>
     </row>
     <row r="21" ht="62" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>US20</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>System Quality and Data Reliability</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Keep decisions traceable</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>As a stakeholder
 I want recruitment decisions to be traceable
 So that the process is transparent and auditable.</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F21" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="F21" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>1. Recruitment decisions must be recorded in a structured way.
 2. Stored decision records must remain accessible when the record is reopened.
-3. The system must preserve enough information to explain the recruitment outcome later.</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="I21" s="6" t="inlineStr">
+3. The system must preserve enough information for later internal review.</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Cross-cutting requirement: traceable records</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J21" s="10" t="inlineStr">
         <is>
           <t>Yifu Feng, Tao Li</t>
         </is>
       </c>
-      <c r="K21" s="8" t="n">
+      <c r="K21" s="11" t="n">
         <v>46125</v>
       </c>
-      <c r="L21" s="8" t="n">
+      <c r="L21" s="11" t="n">
         <v>46145</v>
+      </c>
+    </row>
+    <row r="22" ht="62" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>US21</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Vacancy Posting and Applicant Review</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Add review notes</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>As a module organiser
+I want to add optional review notes or short outcome feedback
+So that recruitment decisions are more transparent and easier to explain later.</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>1. The module organiser must be able to add optional notes when reviewing an application.
+2. Notes must be stored with the application record.
+3. The system must allow the organiser to leave the notes field empty if no extra comment is needed.</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>MO requirement: optional review notes and lightweight feedback</t>
+        </is>
+      </c>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>Tao Li, Chensiyuan Qing</t>
+        </is>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>46125</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="23" ht="62" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>US22</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Applicant Profile and Application</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Show optional outcome feedback</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>As an applicant
+I want to see optional short feedback when it is available
+So that I have slightly more transparency about the recruitment outcome.</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>1. If a module organiser has added a short note that is suitable to share, the applicant must be able to view it with the final outcome.
+2. The system must still work correctly when no feedback note exists.
+3. The first version does not require detailed personalised explanations for every rejection.</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>Applicant requirement: optional outcome feedback</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>Tao Li, Mu Du</t>
+        </is>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>46125</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="24" ht="62" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>US23</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Applicant Profile and Application</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Show applicant count for a vacancy</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>As an applicant
+I want to see how many people have already applied for a vacancy
+So that I have more transparency when deciding whether to apply.</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>1. The system must show the current number of submitted applications for a vacancy when this information is enabled.
+2. The displayed number must match the stored application records.
+3. The vacancy details view must still work correctly when the count is zero.</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>Applicant requirement: application volume transparency</t>
+        </is>
+      </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>Yifu Feng, Tao Li</t>
+        </is>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>46125</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="25" ht="62" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>US24</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Applicant Profile and Application</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Log in from the public interface</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>As a user
+I want to log in from the public vacancy interface with my authorised account
+So that I can access the correct applicant, module organiser, or admin functions when I need protected actions.</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>1. Valid applicant, MO, and admin users must be able to log in from the public interface with credentials.
+2. Invalid credentials must be rejected with a clear message.
+3. Successful login must open the correct role-specific or protected view.
+4. Unauthenticated users may still browse public vacancies but must not access protected functions.</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>Cross-cutting requirement: public browsing and protected login</t>
+        </is>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>Yifu Feng, Mu Du</t>
+        </is>
+      </c>
+      <c r="K25" s="12" t="n">
+        <v>46104</v>
+      </c>
+      <c r="L25" s="12" t="n">
+        <v>46124</v>
+      </c>
+    </row>
+    <row r="26" ht="62" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>US25</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Admin Workload Monitoring</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Configure max_workload parameter</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>As an admin user
+I want to configure the maximum number of roles an applicant can select or apply for
+So that workload control is enforced before manual balancing is needed.</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>1. The admin must be able to set a `max_workload` parameter.
+2. The initial default value can be `3`, but the parameter must be editable.
+3. The system must use the same parameter when checking new applications and showing workload warnings.
+4. The current limit must be shown clearly where it affects user decisions.</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>Admin requirement: configurable workload limit</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t>Yifu Feng, Mu Du</t>
+        </is>
+      </c>
+      <c r="K26" s="12" t="n">
+        <v>46104</v>
+      </c>
+      <c r="L26" s="12" t="n">
+        <v>46124</v>
+      </c>
+    </row>
+    <row r="27" ht="62" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>US26</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Admin Workload Monitoring</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Manage blacklist for unsuitable applicants</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>As an admin user
+I want to maintain a blacklist of unsuitable applicants
+So that students with poor previous performance are not rehired automatically.</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>1. The admin must be able to add or remove blacklist entries.
+2. A blacklist entry should store the applicant identity and a short note or reason.
+3. Blacklisted applicants must be flagged during review or blocked from receiving a new offer according to the policy.
+4. Blacklist records must persist between sessions.</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>Admin requirement: blacklist policy support</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>Mu Du, Chensiyuan Qing</t>
+        </is>
+      </c>
+      <c r="K27" s="12" t="n">
+        <v>46125</v>
+      </c>
+      <c r="L27" s="12" t="n">
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="28" ht="62" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>US27</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Explainable and AI-assisted Enhancements</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Match skills between jobs and applicants</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>As a module organiser
+I want the system to compare vacancy requirements with applicant skills
+So that I can review candidates more efficiently.</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>1. The system should compare structured vacancy requirements with structured applicant skills.
+2. The result should show matched skills or a simple matching score.
+3. The result should be explainable from the stored data rather than opaque.</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>Low-priority explainable AI feature: skill matching</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>Tao Li, Chensiyuan Qing</t>
+        </is>
+      </c>
+      <c r="K28" s="12" t="n">
+        <v>46146</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>46166</v>
+      </c>
+    </row>
+    <row r="29" ht="62" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>US28</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Explainable and AI-assisted Enhancements</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Identify missing skills for applicants</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>As an applicant
+I want to see which skills I am missing for a vacancy
+So that I can decide whether to apply or improve future qualifications.</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>1. The system should list missing or unmatched skills relative to a vacancy.
+2. The explanation should be simple and readable.
+3. The feature should still behave safely when vacancy or profile skill data is incomplete.</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>Low-priority explainable AI feature: missing-skill identification</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>Fuhe Huang, Tao Li</t>
+        </is>
+      </c>
+      <c r="K29" s="12" t="n">
+        <v>46146</v>
+      </c>
+      <c r="L29" s="12" t="n">
+        <v>46166</v>
+      </c>
+    </row>
+    <row r="30" ht="62" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>US29</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Explainable and AI-assisted Enhancements</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Suggest workload balancing</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>As an admin user
+I want the system to suggest workload balancing options
+So that overload risk can be reduced more efficiently.</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>1. The system should suggest possible balancing actions based on current workload data and the max_workload parameter.
+2. The output must be advisory rather than automatic.
+3. The system must still work correctly when no recommendation is available.</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>Low-priority explainable AI feature: workload balancing</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>Mu Du, Yifu Feng</t>
+        </is>
+      </c>
+      <c r="K30" s="12" t="n">
+        <v>46146</v>
+      </c>
+      <c r="L30" s="12" t="n">
+        <v>46166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>